<commit_message>
Vencimentos: recalcula operadores com a correção do bug de pouso em milhar
Regenera base_vencimentos_operadores.xlsx com o parser corrigido (commit
anterior, f35e2459) — valores tipo "1.500" pousos que viravam 1.5 agora
ficam 1500, corrigindo itens que apareciam errado na aba "Próximos".
</commit_message>
<xml_diff>
--- a/Coordenadoria/02_Dados_Tratados/base_vencimentos_operadores.xlsx
+++ b/Coordenadoria/02_Dados_Tratados/base_vencimentos_operadores.xlsx
@@ -20627,7 +20627,7 @@
         <v>886</v>
       </c>
       <c r="K463">
-        <v>26.869</v>
+        <v>26869</v>
       </c>
       <c r="N463" t="b">
         <v>0</v>
@@ -20726,7 +20726,7 @@
         <v>886</v>
       </c>
       <c r="K466">
-        <v>9.082000000000001</v>
+        <v>9082</v>
       </c>
       <c r="N466" t="b">
         <v>0</v>
@@ -20758,7 +20758,7 @@
         <v>886</v>
       </c>
       <c r="K467">
-        <v>10.369</v>
+        <v>10369</v>
       </c>
       <c r="N467" t="b">
         <v>0</v>
@@ -20790,7 +20790,7 @@
         <v>886</v>
       </c>
       <c r="K468">
-        <v>34.566</v>
+        <v>34566</v>
       </c>
       <c r="N468" t="b">
         <v>0</v>
@@ -20822,7 +20822,7 @@
         <v>886</v>
       </c>
       <c r="K469">
-        <v>34.566</v>
+        <v>34566</v>
       </c>
       <c r="N469" t="b">
         <v>0</v>
@@ -20854,7 +20854,7 @@
         <v>886</v>
       </c>
       <c r="K470">
-        <v>36.652</v>
+        <v>36652</v>
       </c>
       <c r="N470" t="b">
         <v>0</v>
@@ -20886,7 +20886,7 @@
         <v>886</v>
       </c>
       <c r="K471">
-        <v>1.714</v>
+        <v>1714</v>
       </c>
       <c r="N471" t="b">
         <v>0</v>
@@ -20918,7 +20918,7 @@
         <v>886</v>
       </c>
       <c r="K472">
-        <v>1.714</v>
+        <v>1714</v>
       </c>
       <c r="N472" t="b">
         <v>0</v>
@@ -21014,7 +21014,7 @@
         <v>886</v>
       </c>
       <c r="K475">
-        <v>1.542</v>
+        <v>1542</v>
       </c>
       <c r="N475" t="b">
         <v>0</v>
@@ -21046,7 +21046,7 @@
         <v>886</v>
       </c>
       <c r="K476">
-        <v>1.542</v>
+        <v>1542</v>
       </c>
       <c r="N476" t="b">
         <v>0</v>
@@ -21078,7 +21078,7 @@
         <v>886</v>
       </c>
       <c r="K477">
-        <v>17.488</v>
+        <v>17488</v>
       </c>
       <c r="N477" t="b">
         <v>0</v>
@@ -21110,7 +21110,7 @@
         <v>886</v>
       </c>
       <c r="K478">
-        <v>21.139</v>
+        <v>21139</v>
       </c>
       <c r="N478" t="b">
         <v>0</v>
@@ -21142,7 +21142,7 @@
         <v>886</v>
       </c>
       <c r="K479">
-        <v>21.139</v>
+        <v>21139</v>
       </c>
       <c r="N479" t="b">
         <v>0</v>
@@ -21174,7 +21174,7 @@
         <v>886</v>
       </c>
       <c r="K480">
-        <v>17.488</v>
+        <v>17488</v>
       </c>
       <c r="N480" t="b">
         <v>0</v>
@@ -21206,7 +21206,7 @@
         <v>886</v>
       </c>
       <c r="K481">
-        <v>17.488</v>
+        <v>17488</v>
       </c>
       <c r="N481" t="b">
         <v>0</v>
@@ -21238,7 +21238,7 @@
         <v>886</v>
       </c>
       <c r="K482">
-        <v>17.488</v>
+        <v>17488</v>
       </c>
       <c r="N482" t="b">
         <v>0</v>
@@ -21270,7 +21270,7 @@
         <v>886</v>
       </c>
       <c r="K483">
-        <v>17.488</v>
+        <v>17488</v>
       </c>
       <c r="N483" t="b">
         <v>0</v>
@@ -21302,7 +21302,7 @@
         <v>886</v>
       </c>
       <c r="K484">
-        <v>21.603</v>
+        <v>21603</v>
       </c>
       <c r="N484" t="b">
         <v>0</v>
@@ -21334,7 +21334,7 @@
         <v>886</v>
       </c>
       <c r="K485">
-        <v>21.603</v>
+        <v>21603</v>
       </c>
       <c r="N485" t="b">
         <v>0</v>
@@ -21366,7 +21366,7 @@
         <v>886</v>
       </c>
       <c r="K486">
-        <v>27.308</v>
+        <v>27308</v>
       </c>
       <c r="N486" t="b">
         <v>0</v>
@@ -21398,7 +21398,7 @@
         <v>886</v>
       </c>
       <c r="K487">
-        <v>4.95</v>
+        <v>4950</v>
       </c>
       <c r="N487" t="b">
         <v>0</v>
@@ -21462,7 +21462,7 @@
         <v>886</v>
       </c>
       <c r="K489">
-        <v>4.303</v>
+        <v>4303</v>
       </c>
       <c r="N489" t="b">
         <v>0</v>
@@ -21494,7 +21494,7 @@
         <v>886</v>
       </c>
       <c r="K490">
-        <v>2.195</v>
+        <v>2195</v>
       </c>
       <c r="N490" t="b">
         <v>0</v>
@@ -21526,7 +21526,7 @@
         <v>886</v>
       </c>
       <c r="K491">
-        <v>27.195</v>
+        <v>27195</v>
       </c>
       <c r="N491" t="b">
         <v>0</v>
@@ -21558,7 +21558,7 @@
         <v>886</v>
       </c>
       <c r="K492">
-        <v>27.172</v>
+        <v>27172</v>
       </c>
       <c r="N492" t="b">
         <v>0</v>
@@ -21590,7 +21590,7 @@
         <v>886</v>
       </c>
       <c r="K493">
-        <v>35.808</v>
+        <v>35808</v>
       </c>
       <c r="N493" t="b">
         <v>0</v>
@@ -21756,7 +21756,7 @@
         <v>886</v>
       </c>
       <c r="K498">
-        <v>1.019</v>
+        <v>1019</v>
       </c>
       <c r="N498" t="b">
         <v>0</v>
@@ -21788,7 +21788,7 @@
         <v>886</v>
       </c>
       <c r="K499">
-        <v>1.019</v>
+        <v>1019</v>
       </c>
       <c r="N499" t="b">
         <v>0</v>
@@ -21820,7 +21820,7 @@
         <v>886</v>
       </c>
       <c r="K500">
-        <v>26.036</v>
+        <v>26036</v>
       </c>
       <c r="N500" t="b">
         <v>0</v>
@@ -21852,7 +21852,7 @@
         <v>886</v>
       </c>
       <c r="K501">
-        <v>26.036</v>
+        <v>26036</v>
       </c>
       <c r="N501" t="b">
         <v>0</v>
@@ -21884,7 +21884,7 @@
         <v>886</v>
       </c>
       <c r="K502">
-        <v>26.036</v>
+        <v>26036</v>
       </c>
       <c r="N502" t="b">
         <v>0</v>
@@ -21916,7 +21916,7 @@
         <v>886</v>
       </c>
       <c r="K503">
-        <v>26.036</v>
+        <v>26036</v>
       </c>
       <c r="N503" t="b">
         <v>0</v>
@@ -21948,7 +21948,7 @@
         <v>886</v>
       </c>
       <c r="K504">
-        <v>28.898</v>
+        <v>28898</v>
       </c>
       <c r="N504" t="b">
         <v>0</v>
@@ -21980,7 +21980,7 @@
         <v>886</v>
       </c>
       <c r="K505">
-        <v>27.308</v>
+        <v>27308</v>
       </c>
       <c r="N505" t="b">
         <v>0</v>
@@ -22012,7 +22012,7 @@
         <v>886</v>
       </c>
       <c r="K506">
-        <v>27.308</v>
+        <v>27308</v>
       </c>
       <c r="N506" t="b">
         <v>0</v>
@@ -22044,7 +22044,7 @@
         <v>886</v>
       </c>
       <c r="K507">
-        <v>26.334</v>
+        <v>26334</v>
       </c>
       <c r="N507" t="b">
         <v>0</v>
@@ -22076,7 +22076,7 @@
         <v>886</v>
       </c>
       <c r="K508">
-        <v>26.334</v>
+        <v>26334</v>
       </c>
       <c r="N508" t="b">
         <v>0</v>
@@ -22108,7 +22108,7 @@
         <v>886</v>
       </c>
       <c r="K509">
-        <v>5.289</v>
+        <v>5289</v>
       </c>
       <c r="N509" t="b">
         <v>0</v>
@@ -22140,7 +22140,7 @@
         <v>886</v>
       </c>
       <c r="K510">
-        <v>30.286</v>
+        <v>30286</v>
       </c>
       <c r="N510" t="b">
         <v>0</v>
@@ -22172,7 +22172,7 @@
         <v>886</v>
       </c>
       <c r="K511">
-        <v>30.286</v>
+        <v>30286</v>
       </c>
       <c r="N511" t="b">
         <v>0</v>
@@ -22204,7 +22204,7 @@
         <v>886</v>
       </c>
       <c r="K512">
-        <v>30.286</v>
+        <v>30286</v>
       </c>
       <c r="N512" t="b">
         <v>0</v>
@@ -22392,7 +22392,7 @@
         <v>886</v>
       </c>
       <c r="K519">
-        <v>21.664</v>
+        <v>21664</v>
       </c>
       <c r="N519" t="b">
         <v>0</v>
@@ -22424,7 +22424,7 @@
         <v>886</v>
       </c>
       <c r="K520">
-        <v>27.957</v>
+        <v>27957</v>
       </c>
       <c r="N520" t="b">
         <v>0</v>
@@ -22456,7 +22456,7 @@
         <v>886</v>
       </c>
       <c r="K521">
-        <v>26.963</v>
+        <v>26963</v>
       </c>
       <c r="N521" t="b">
         <v>0</v>
@@ -22488,7 +22488,7 @@
         <v>886</v>
       </c>
       <c r="K522">
-        <v>29.113</v>
+        <v>29113</v>
       </c>
       <c r="N522" t="b">
         <v>0</v>
@@ -22520,7 +22520,7 @@
         <v>886</v>
       </c>
       <c r="K523">
-        <v>29.113</v>
+        <v>29113</v>
       </c>
       <c r="N523" t="b">
         <v>0</v>
@@ -22552,7 +22552,7 @@
         <v>886</v>
       </c>
       <c r="K524">
-        <v>29.113</v>
+        <v>29113</v>
       </c>
       <c r="N524" t="b">
         <v>0</v>
@@ -22584,7 +22584,7 @@
         <v>886</v>
       </c>
       <c r="K525">
-        <v>29.113</v>
+        <v>29113</v>
       </c>
       <c r="N525" t="b">
         <v>0</v>
@@ -22616,7 +22616,7 @@
         <v>886</v>
       </c>
       <c r="K526">
-        <v>22.121</v>
+        <v>22121</v>
       </c>
       <c r="N526" t="b">
         <v>0</v>
@@ -22648,7 +22648,7 @@
         <v>886</v>
       </c>
       <c r="K527">
-        <v>22.121</v>
+        <v>22121</v>
       </c>
       <c r="N527" t="b">
         <v>0</v>
@@ -22680,7 +22680,7 @@
         <v>886</v>
       </c>
       <c r="K528">
-        <v>22.83</v>
+        <v>22830</v>
       </c>
       <c r="N528" t="b">
         <v>0</v>
@@ -22776,7 +22776,7 @@
         <v>886</v>
       </c>
       <c r="K531">
-        <v>6.074</v>
+        <v>6074</v>
       </c>
       <c r="N531" t="b">
         <v>0</v>
@@ -22808,7 +22808,7 @@
         <v>886</v>
       </c>
       <c r="K532">
-        <v>4.566</v>
+        <v>4566</v>
       </c>
       <c r="N532" t="b">
         <v>0</v>
@@ -22840,7 +22840,7 @@
         <v>886</v>
       </c>
       <c r="K533">
-        <v>23.095</v>
+        <v>23095</v>
       </c>
       <c r="N533" t="b">
         <v>0</v>
@@ -22872,7 +22872,7 @@
         <v>886</v>
       </c>
       <c r="K534">
-        <v>28.281</v>
+        <v>28281</v>
       </c>
       <c r="N534" t="b">
         <v>0</v>
@@ -22904,7 +22904,7 @@
         <v>886</v>
       </c>
       <c r="K535">
-        <v>28.281</v>
+        <v>28281</v>
       </c>
       <c r="N535" t="b">
         <v>0</v>
@@ -23128,7 +23128,7 @@
         <v>886</v>
       </c>
       <c r="K542">
-        <v>23.393</v>
+        <v>23393</v>
       </c>
       <c r="N542" t="b">
         <v>0</v>
@@ -23160,7 +23160,7 @@
         <v>886</v>
       </c>
       <c r="K543">
-        <v>23.393</v>
+        <v>23393</v>
       </c>
       <c r="N543" t="b">
         <v>0</v>
@@ -23192,7 +23192,7 @@
         <v>886</v>
       </c>
       <c r="K544">
-        <v>23.393</v>
+        <v>23393</v>
       </c>
       <c r="N544" t="b">
         <v>0</v>
@@ -23224,7 +23224,7 @@
         <v>886</v>
       </c>
       <c r="K545">
-        <v>22.83</v>
+        <v>22830</v>
       </c>
       <c r="N545" t="b">
         <v>0</v>
@@ -23256,7 +23256,7 @@
         <v>886</v>
       </c>
       <c r="K546">
-        <v>22.83</v>
+        <v>22830</v>
       </c>
       <c r="N546" t="b">
         <v>0</v>
@@ -23288,7 +23288,7 @@
         <v>886</v>
       </c>
       <c r="K547">
-        <v>22.83</v>
+        <v>22830</v>
       </c>
       <c r="N547" t="b">
         <v>0</v>
@@ -23320,7 +23320,7 @@
         <v>886</v>
       </c>
       <c r="K548">
-        <v>22.83</v>
+        <v>22830</v>
       </c>
       <c r="N548" t="b">
         <v>0</v>
@@ -23352,7 +23352,7 @@
         <v>886</v>
       </c>
       <c r="K549">
-        <v>22.83</v>
+        <v>22830</v>
       </c>
       <c r="N549" t="b">
         <v>0</v>
@@ -23384,7 +23384,7 @@
         <v>886</v>
       </c>
       <c r="K550">
-        <v>22.83</v>
+        <v>22830</v>
       </c>
       <c r="N550" t="b">
         <v>0</v>
@@ -23416,7 +23416,7 @@
         <v>886</v>
       </c>
       <c r="K551">
-        <v>27.284</v>
+        <v>27284</v>
       </c>
       <c r="N551" t="b">
         <v>0</v>
@@ -23448,7 +23448,7 @@
         <v>886</v>
       </c>
       <c r="K552">
-        <v>3.884</v>
+        <v>3884</v>
       </c>
       <c r="N552" t="b">
         <v>0</v>
@@ -23480,7 +23480,7 @@
         <v>886</v>
       </c>
       <c r="K553">
-        <v>3.328</v>
+        <v>3328</v>
       </c>
       <c r="N553" t="b">
         <v>0</v>
@@ -23512,7 +23512,7 @@
         <v>886</v>
       </c>
       <c r="K554">
-        <v>4.089</v>
+        <v>4089</v>
       </c>
       <c r="N554" t="b">
         <v>0</v>
@@ -23544,7 +23544,7 @@
         <v>886</v>
       </c>
       <c r="K555">
-        <v>5.878</v>
+        <v>5878</v>
       </c>
       <c r="N555" t="b">
         <v>0</v>
@@ -23576,7 +23576,7 @@
         <v>886</v>
       </c>
       <c r="K556">
-        <v>30.878</v>
+        <v>30878</v>
       </c>
       <c r="N556" t="b">
         <v>0</v>
@@ -23608,7 +23608,7 @@
         <v>886</v>
       </c>
       <c r="K557">
-        <v>33.602</v>
+        <v>33602</v>
       </c>
       <c r="N557" t="b">
         <v>0</v>
@@ -23640,7 +23640,7 @@
         <v>886</v>
       </c>
       <c r="K558">
-        <v>30.878</v>
+        <v>30878</v>
       </c>
       <c r="N558" t="b">
         <v>0</v>
@@ -23870,7 +23870,7 @@
         <v>886</v>
       </c>
       <c r="K565">
-        <v>21.853</v>
+        <v>21853</v>
       </c>
       <c r="N565" t="b">
         <v>0</v>
@@ -23902,7 +23902,7 @@
         <v>886</v>
       </c>
       <c r="K566">
-        <v>21.617</v>
+        <v>21617</v>
       </c>
       <c r="N566" t="b">
         <v>0</v>
@@ -23934,7 +23934,7 @@
         <v>886</v>
       </c>
       <c r="K567">
-        <v>24.088</v>
+        <v>24088</v>
       </c>
       <c r="N567" t="b">
         <v>0</v>
@@ -23966,7 +23966,7 @@
         <v>886</v>
       </c>
       <c r="K568">
-        <v>30.369</v>
+        <v>30369</v>
       </c>
       <c r="N568" t="b">
         <v>0</v>
@@ -23998,7 +23998,7 @@
         <v>886</v>
       </c>
       <c r="K569">
-        <v>23.846</v>
+        <v>23846</v>
       </c>
       <c r="N569" t="b">
         <v>0</v>
@@ -24030,7 +24030,7 @@
         <v>886</v>
       </c>
       <c r="K570">
-        <v>29.26</v>
+        <v>29260</v>
       </c>
       <c r="N570" t="b">
         <v>0</v>
@@ -24062,7 +24062,7 @@
         <v>886</v>
       </c>
       <c r="K571">
-        <v>25.113</v>
+        <v>25113</v>
       </c>
       <c r="N571" t="b">
         <v>0</v>
@@ -24094,7 +24094,7 @@
         <v>886</v>
       </c>
       <c r="K572">
-        <v>14.914</v>
+        <v>14914</v>
       </c>
       <c r="N572" t="b">
         <v>0</v>
@@ -24126,7 +24126,7 @@
         <v>886</v>
       </c>
       <c r="K573">
-        <v>14.914</v>
+        <v>14914</v>
       </c>
       <c r="N573" t="b">
         <v>0</v>
@@ -24222,7 +24222,7 @@
         <v>886</v>
       </c>
       <c r="K576">
-        <v>9.768000000000001</v>
+        <v>9768</v>
       </c>
       <c r="N576" t="b">
         <v>0</v>
@@ -24254,7 +24254,7 @@
         <v>886</v>
       </c>
       <c r="K577">
-        <v>12.861</v>
+        <v>12861</v>
       </c>
       <c r="N577" t="b">
         <v>0</v>
@@ -24286,7 +24286,7 @@
         <v>886</v>
       </c>
       <c r="K578">
-        <v>31.717</v>
+        <v>31717</v>
       </c>
       <c r="N578" t="b">
         <v>0</v>
@@ -24318,7 +24318,7 @@
         <v>886</v>
       </c>
       <c r="K579">
-        <v>31.717</v>
+        <v>31717</v>
       </c>
       <c r="N579" t="b">
         <v>0</v>
@@ -24350,7 +24350,7 @@
         <v>886</v>
       </c>
       <c r="K580">
-        <v>31.155</v>
+        <v>31155</v>
       </c>
       <c r="N580" t="b">
         <v>0</v>
@@ -24382,7 +24382,7 @@
         <v>886</v>
       </c>
       <c r="K581">
-        <v>1.717</v>
+        <v>1717</v>
       </c>
       <c r="N581" t="b">
         <v>0</v>
@@ -24478,7 +24478,7 @@
         <v>886</v>
       </c>
       <c r="K584">
-        <v>1.93</v>
+        <v>1930</v>
       </c>
       <c r="N584" t="b">
         <v>0</v>
@@ -24510,7 +24510,7 @@
         <v>886</v>
       </c>
       <c r="K585">
-        <v>1.768</v>
+        <v>1768</v>
       </c>
       <c r="N585" t="b">
         <v>0</v>
@@ -24542,7 +24542,7 @@
         <v>886</v>
       </c>
       <c r="K586">
-        <v>1.768</v>
+        <v>1768</v>
       </c>
       <c r="N586" t="b">
         <v>0</v>
@@ -24574,7 +24574,7 @@
         <v>886</v>
       </c>
       <c r="K587">
-        <v>25.181</v>
+        <v>25181</v>
       </c>
       <c r="N587" t="b">
         <v>0</v>
@@ -24606,7 +24606,7 @@
         <v>886</v>
       </c>
       <c r="K588">
-        <v>25.175</v>
+        <v>25175</v>
       </c>
       <c r="N588" t="b">
         <v>0</v>
@@ -24638,7 +24638,7 @@
         <v>886</v>
       </c>
       <c r="K589">
-        <v>25.175</v>
+        <v>25175</v>
       </c>
       <c r="N589" t="b">
         <v>0</v>
@@ -24670,7 +24670,7 @@
         <v>886</v>
       </c>
       <c r="K590">
-        <v>23.819</v>
+        <v>23819</v>
       </c>
       <c r="N590" t="b">
         <v>0</v>
@@ -24702,7 +24702,7 @@
         <v>886</v>
       </c>
       <c r="K591">
-        <v>31.268</v>
+        <v>31268</v>
       </c>
       <c r="N591" t="b">
         <v>0</v>
@@ -24734,7 +24734,7 @@
         <v>886</v>
       </c>
       <c r="K592">
-        <v>18.925</v>
+        <v>18925</v>
       </c>
       <c r="N592" t="b">
         <v>0</v>
@@ -24766,7 +24766,7 @@
         <v>886</v>
       </c>
       <c r="K593">
-        <v>26.151</v>
+        <v>26151</v>
       </c>
       <c r="N593" t="b">
         <v>0</v>
@@ -24798,7 +24798,7 @@
         <v>886</v>
       </c>
       <c r="K594">
-        <v>23.811</v>
+        <v>23811</v>
       </c>
       <c r="N594" t="b">
         <v>0</v>
@@ -24830,7 +24830,7 @@
         <v>886</v>
       </c>
       <c r="K595">
-        <v>24.268</v>
+        <v>24268</v>
       </c>
       <c r="N595" t="b">
         <v>0</v>
@@ -24862,7 +24862,7 @@
         <v>886</v>
       </c>
       <c r="K596">
-        <v>25.431</v>
+        <v>25431</v>
       </c>
       <c r="N596" t="b">
         <v>0</v>
@@ -24961,7 +24961,7 @@
         <v>886</v>
       </c>
       <c r="K599">
-        <v>8.542999999999999</v>
+        <v>8543</v>
       </c>
       <c r="N599" t="b">
         <v>0</v>
@@ -24993,7 +24993,7 @@
         <v>886</v>
       </c>
       <c r="K600">
-        <v>3.934</v>
+        <v>3934</v>
       </c>
       <c r="N600" t="b">
         <v>0</v>
@@ -25022,7 +25022,7 @@
         <v>886</v>
       </c>
       <c r="K601">
-        <v>28.934</v>
+        <v>28934</v>
       </c>
       <c r="N601" t="b">
         <v>0</v>
@@ -25051,7 +25051,7 @@
         <v>886</v>
       </c>
       <c r="K602">
-        <v>28.934</v>
+        <v>28934</v>
       </c>
       <c r="N602" t="b">
         <v>0</v>
@@ -25080,7 +25080,7 @@
         <v>886</v>
       </c>
       <c r="K603">
-        <v>28.934</v>
+        <v>28934</v>
       </c>
       <c r="N603" t="b">
         <v>0</v>
@@ -25112,7 +25112,7 @@
         <v>886</v>
       </c>
       <c r="K604">
-        <v>1.501</v>
+        <v>1501</v>
       </c>
       <c r="N604" t="b">
         <v>0</v>
@@ -25144,7 +25144,7 @@
         <v>886</v>
       </c>
       <c r="K605">
-        <v>1.501</v>
+        <v>1501</v>
       </c>
       <c r="N605" t="b">
         <v>0</v>
@@ -25176,7 +25176,7 @@
         <v>886</v>
       </c>
       <c r="K606">
-        <v>1.484</v>
+        <v>1484</v>
       </c>
       <c r="N606" t="b">
         <v>0</v>
@@ -25208,7 +25208,7 @@
         <v>886</v>
       </c>
       <c r="K607">
-        <v>1.484</v>
+        <v>1484</v>
       </c>
       <c r="N607" t="b">
         <v>0</v>
@@ -25240,7 +25240,7 @@
         <v>886</v>
       </c>
       <c r="K608">
-        <v>1.484</v>
+        <v>1484</v>
       </c>
       <c r="N608" t="b">
         <v>0</v>
@@ -25272,7 +25272,7 @@
         <v>886</v>
       </c>
       <c r="K609">
-        <v>1.484</v>
+        <v>1484</v>
       </c>
       <c r="N609" t="b">
         <v>0</v>
@@ -25304,7 +25304,7 @@
         <v>886</v>
       </c>
       <c r="K610">
-        <v>25.431</v>
+        <v>25431</v>
       </c>
       <c r="N610" t="b">
         <v>0</v>
@@ -25336,7 +25336,7 @@
         <v>886</v>
       </c>
       <c r="K611">
-        <v>25.431</v>
+        <v>25431</v>
       </c>
       <c r="N611" t="b">
         <v>0</v>
@@ -25368,7 +25368,7 @@
         <v>886</v>
       </c>
       <c r="K612">
-        <v>25.431</v>
+        <v>25431</v>
       </c>
       <c r="N612" t="b">
         <v>0</v>
@@ -25400,7 +25400,7 @@
         <v>886</v>
       </c>
       <c r="K613">
-        <v>25.431</v>
+        <v>25431</v>
       </c>
       <c r="N613" t="b">
         <v>0</v>
@@ -25432,7 +25432,7 @@
         <v>886</v>
       </c>
       <c r="K614">
-        <v>29.952</v>
+        <v>29952</v>
       </c>
       <c r="N614" t="b">
         <v>0</v>
@@ -25464,7 +25464,7 @@
         <v>886</v>
       </c>
       <c r="K615">
-        <v>25.431</v>
+        <v>25431</v>
       </c>
       <c r="N615" t="b">
         <v>0</v>
@@ -25496,7 +25496,7 @@
         <v>886</v>
       </c>
       <c r="K616">
-        <v>25.431</v>
+        <v>25431</v>
       </c>
       <c r="N616" t="b">
         <v>0</v>
@@ -25528,7 +25528,7 @@
         <v>886</v>
       </c>
       <c r="K617">
-        <v>25.431</v>
+        <v>25431</v>
       </c>
       <c r="N617" t="b">
         <v>0</v>
@@ -25560,7 +25560,7 @@
         <v>886</v>
       </c>
       <c r="K618">
-        <v>25.431</v>
+        <v>25431</v>
       </c>
       <c r="N618" t="b">
         <v>0</v>
@@ -25592,7 +25592,7 @@
         <v>886</v>
       </c>
       <c r="K619">
-        <v>26.511</v>
+        <v>26511</v>
       </c>
       <c r="N619" t="b">
         <v>0</v>
@@ -25656,7 +25656,7 @@
         <v>886</v>
       </c>
       <c r="K621">
-        <v>4.091</v>
+        <v>4091</v>
       </c>
       <c r="N621" t="b">
         <v>0</v>
@@ -25688,7 +25688,7 @@
         <v>886</v>
       </c>
       <c r="K622">
-        <v>9.68</v>
+        <v>9680</v>
       </c>
       <c r="N622" t="b">
         <v>0</v>
@@ -25720,7 +25720,7 @@
         <v>886</v>
       </c>
       <c r="K623">
-        <v>7.048</v>
+        <v>7048</v>
       </c>
       <c r="N623" t="b">
         <v>0</v>
@@ -25752,7 +25752,7 @@
         <v>886</v>
       </c>
       <c r="K624">
-        <v>39.68</v>
+        <v>39680</v>
       </c>
       <c r="N624" t="b">
         <v>0</v>
@@ -25784,7 +25784,7 @@
         <v>886</v>
       </c>
       <c r="K625">
-        <v>32.048</v>
+        <v>32048</v>
       </c>
       <c r="N625" t="b">
         <v>0</v>
@@ -25816,7 +25816,7 @@
         <v>886</v>
       </c>
       <c r="K626">
-        <v>32.048</v>
+        <v>32048</v>
       </c>
       <c r="N626" t="b">
         <v>0</v>
@@ -25848,7 +25848,7 @@
         <v>886</v>
       </c>
       <c r="K627">
-        <v>1.803</v>
+        <v>1803</v>
       </c>
       <c r="N627" t="b">
         <v>0</v>
@@ -25912,7 +25912,7 @@
         <v>886</v>
       </c>
       <c r="K629">
-        <v>1.52</v>
+        <v>1520</v>
       </c>
       <c r="N629" t="b">
         <v>0</v>
@@ -25944,7 +25944,7 @@
         <v>886</v>
       </c>
       <c r="K630">
-        <v>1.52</v>
+        <v>1520</v>
       </c>
       <c r="N630" t="b">
         <v>0</v>
@@ -26040,7 +26040,7 @@
         <v>886</v>
       </c>
       <c r="K633">
-        <v>28.073</v>
+        <v>28073</v>
       </c>
       <c r="N633" t="b">
         <v>0</v>
@@ -26072,7 +26072,7 @@
         <v>886</v>
       </c>
       <c r="K634">
-        <v>24.089</v>
+        <v>24089</v>
       </c>
       <c r="N634" t="b">
         <v>0</v>
@@ -26104,7 +26104,7 @@
         <v>886</v>
       </c>
       <c r="K635">
-        <v>24.093</v>
+        <v>24093</v>
       </c>
       <c r="N635" t="b">
         <v>0</v>
@@ -26136,7 +26136,7 @@
         <v>886</v>
       </c>
       <c r="K636">
-        <v>29.002</v>
+        <v>29002</v>
       </c>
       <c r="N636" t="b">
         <v>0</v>
@@ -26168,7 +26168,7 @@
         <v>886</v>
       </c>
       <c r="K637">
-        <v>31.303</v>
+        <v>31303</v>
       </c>
       <c r="N637" t="b">
         <v>0</v>
@@ -26200,7 +26200,7 @@
         <v>886</v>
       </c>
       <c r="K638">
-        <v>29.002</v>
+        <v>29002</v>
       </c>
       <c r="N638" t="b">
         <v>0</v>
@@ -26232,7 +26232,7 @@
         <v>886</v>
       </c>
       <c r="K639">
-        <v>29.002</v>
+        <v>29002</v>
       </c>
       <c r="N639" t="b">
         <v>0</v>
@@ -26264,7 +26264,7 @@
         <v>886</v>
       </c>
       <c r="K640">
-        <v>29.37</v>
+        <v>29370</v>
       </c>
       <c r="N640" t="b">
         <v>0</v>
@@ -26296,7 +26296,7 @@
         <v>886</v>
       </c>
       <c r="K641">
-        <v>29.37</v>
+        <v>29370</v>
       </c>
       <c r="N641" t="b">
         <v>0</v>
@@ -26363,7 +26363,7 @@
         <v>886</v>
       </c>
       <c r="K643">
-        <v>2.204</v>
+        <v>2204</v>
       </c>
       <c r="N643" t="b">
         <v>0</v>
@@ -26395,7 +26395,7 @@
         <v>886</v>
       </c>
       <c r="K644">
-        <v>8.826000000000001</v>
+        <v>8826</v>
       </c>
       <c r="N644" t="b">
         <v>0</v>
@@ -26427,7 +26427,7 @@
         <v>886</v>
       </c>
       <c r="K645">
-        <v>7.152</v>
+        <v>7152</v>
       </c>
       <c r="N645" t="b">
         <v>0</v>
@@ -26459,7 +26459,7 @@
         <v>886</v>
       </c>
       <c r="K646">
-        <v>39.725</v>
+        <v>39725</v>
       </c>
       <c r="N646" t="b">
         <v>0</v>
@@ -26491,7 +26491,7 @@
         <v>886</v>
       </c>
       <c r="K647">
-        <v>37.725</v>
+        <v>37725</v>
       </c>
       <c r="N647" t="b">
         <v>0</v>
@@ -26523,7 +26523,7 @@
         <v>886</v>
       </c>
       <c r="K648">
-        <v>36.567</v>
+        <v>36567</v>
       </c>
       <c r="N648" t="b">
         <v>0</v>
@@ -26747,7 +26747,7 @@
         <v>886</v>
       </c>
       <c r="K655">
-        <v>25.611</v>
+        <v>25611</v>
       </c>
       <c r="N655" t="b">
         <v>0</v>
@@ -26779,7 +26779,7 @@
         <v>886</v>
       </c>
       <c r="K656">
-        <v>25.611</v>
+        <v>25611</v>
       </c>
       <c r="N656" t="b">
         <v>0</v>
@@ -26811,7 +26811,7 @@
         <v>886</v>
       </c>
       <c r="K657">
-        <v>25.611</v>
+        <v>25611</v>
       </c>
       <c r="N657" t="b">
         <v>0</v>
@@ -26843,7 +26843,7 @@
         <v>886</v>
       </c>
       <c r="K658">
-        <v>30.355</v>
+        <v>30355</v>
       </c>
       <c r="N658" t="b">
         <v>0</v>
@@ -26875,7 +26875,7 @@
         <v>886</v>
       </c>
       <c r="K659">
-        <v>30.355</v>
+        <v>30355</v>
       </c>
       <c r="N659" t="b">
         <v>0</v>
@@ -26907,7 +26907,7 @@
         <v>886</v>
       </c>
       <c r="K660">
-        <v>30.355</v>
+        <v>30355</v>
       </c>
       <c r="N660" t="b">
         <v>0</v>
@@ -26939,7 +26939,7 @@
         <v>886</v>
       </c>
       <c r="K661">
-        <v>30.355</v>
+        <v>30355</v>
       </c>
       <c r="N661" t="b">
         <v>0</v>
@@ -26971,7 +26971,7 @@
         <v>886</v>
       </c>
       <c r="K662">
-        <v>30.269</v>
+        <v>30269</v>
       </c>
       <c r="N662" t="b">
         <v>0</v>
@@ -27003,7 +27003,7 @@
         <v>886</v>
       </c>
       <c r="K663">
-        <v>25.611</v>
+        <v>25611</v>
       </c>
       <c r="N663" t="b">
         <v>0</v>
@@ -27493,7 +27493,7 @@
         <v>886</v>
       </c>
       <c r="K677">
-        <v>34.13</v>
+        <v>34130</v>
       </c>
       <c r="N677" t="b">
         <v>0</v>
@@ -27522,7 +27522,7 @@
         <v>886</v>
       </c>
       <c r="K678">
-        <v>4.13</v>
+        <v>4130</v>
       </c>
       <c r="N678" t="b">
         <v>0</v>
@@ -27551,7 +27551,7 @@
         <v>886</v>
       </c>
       <c r="K679">
-        <v>4.13</v>
+        <v>4130</v>
       </c>
       <c r="N679" t="b">
         <v>0</v>
@@ -27583,7 +27583,7 @@
         <v>886</v>
       </c>
       <c r="K680">
-        <v>4.869</v>
+        <v>4869</v>
       </c>
       <c r="N680" t="b">
         <v>0</v>
@@ -27615,7 +27615,7 @@
         <v>886</v>
       </c>
       <c r="K681">
-        <v>22.46</v>
+        <v>22460</v>
       </c>
       <c r="N681" t="b">
         <v>0</v>
@@ -27790,7 +27790,7 @@
         <v>886</v>
       </c>
       <c r="K686">
-        <v>35.41</v>
+        <v>35410</v>
       </c>
       <c r="N686" t="b">
         <v>0</v>
@@ -27819,7 +27819,7 @@
         <v>886</v>
       </c>
       <c r="K687">
-        <v>5.41</v>
+        <v>5410</v>
       </c>
       <c r="N687" t="b">
         <v>0</v>
@@ -27848,7 +27848,7 @@
         <v>886</v>
       </c>
       <c r="K688">
-        <v>5.41</v>
+        <v>5410</v>
       </c>
       <c r="N688" t="b">
         <v>0</v>
@@ -27880,7 +27880,7 @@
         <v>886</v>
       </c>
       <c r="K689">
-        <v>5.534</v>
+        <v>5534</v>
       </c>
       <c r="N689" t="b">
         <v>0</v>
@@ -27912,7 +27912,7 @@
         <v>886</v>
       </c>
       <c r="K690">
-        <v>35.41</v>
+        <v>35410</v>
       </c>
       <c r="N690" t="b">
         <v>0</v>
@@ -28087,7 +28087,7 @@
         <v>886</v>
       </c>
       <c r="K695">
-        <v>30.286</v>
+        <v>30286</v>
       </c>
       <c r="N695" t="b">
         <v>0</v>
@@ -28119,7 +28119,7 @@
         <v>886</v>
       </c>
       <c r="K696">
-        <v>30.289</v>
+        <v>30289</v>
       </c>
       <c r="N696" t="b">
         <v>0</v>
@@ -28273,7 +28273,7 @@
         <v>886</v>
       </c>
       <c r="K701">
-        <v>33.695</v>
+        <v>33695</v>
       </c>
       <c r="N701" t="b">
         <v>0</v>
@@ -28302,7 +28302,7 @@
         <v>886</v>
       </c>
       <c r="K702">
-        <v>3.695</v>
+        <v>3695</v>
       </c>
       <c r="N702" t="b">
         <v>0</v>
@@ -28331,7 +28331,7 @@
         <v>886</v>
       </c>
       <c r="K703">
-        <v>3.695</v>
+        <v>3695</v>
       </c>
       <c r="N703" t="b">
         <v>0</v>
@@ -28363,7 +28363,7 @@
         <v>886</v>
       </c>
       <c r="K704">
-        <v>4.201</v>
+        <v>4201</v>
       </c>
       <c r="N704" t="b">
         <v>0</v>
@@ -28395,7 +28395,7 @@
         <v>886</v>
       </c>
       <c r="K705">
-        <v>28.281</v>
+        <v>28281</v>
       </c>
       <c r="N705" t="b">
         <v>0</v>
@@ -28570,7 +28570,7 @@
         <v>886</v>
       </c>
       <c r="K710">
-        <v>34.008</v>
+        <v>34008</v>
       </c>
       <c r="N710" t="b">
         <v>0</v>
@@ -28599,7 +28599,7 @@
         <v>886</v>
       </c>
       <c r="K711">
-        <v>4.008</v>
+        <v>4008</v>
       </c>
       <c r="N711" t="b">
         <v>0</v>
@@ -28628,7 +28628,7 @@
         <v>886</v>
       </c>
       <c r="K712">
-        <v>4.008</v>
+        <v>4008</v>
       </c>
       <c r="N712" t="b">
         <v>0</v>
@@ -28660,7 +28660,7 @@
         <v>886</v>
       </c>
       <c r="K713">
-        <v>8.784000000000001</v>
+        <v>8784</v>
       </c>
       <c r="N713" t="b">
         <v>0</v>
@@ -28692,7 +28692,7 @@
         <v>886</v>
       </c>
       <c r="K714">
-        <v>30.233</v>
+        <v>30233</v>
       </c>
       <c r="N714" t="b">
         <v>0</v>
@@ -28829,7 +28829,7 @@
         <v>886</v>
       </c>
       <c r="K718">
-        <v>31.717</v>
+        <v>31717</v>
       </c>
       <c r="N718" t="b">
         <v>0</v>
@@ -28858,7 +28858,7 @@
         <v>886</v>
       </c>
       <c r="K719">
-        <v>1.717</v>
+        <v>1717</v>
       </c>
       <c r="N719" t="b">
         <v>0</v>
@@ -28887,7 +28887,7 @@
         <v>886</v>
       </c>
       <c r="K720">
-        <v>1.717</v>
+        <v>1717</v>
       </c>
       <c r="N720" t="b">
         <v>0</v>
@@ -28919,7 +28919,7 @@
         <v>886</v>
       </c>
       <c r="K721">
-        <v>1.217</v>
+        <v>1217</v>
       </c>
       <c r="N721" t="b">
         <v>0</v>
@@ -28951,7 +28951,7 @@
         <v>886</v>
       </c>
       <c r="K722">
-        <v>31.717</v>
+        <v>31717</v>
       </c>
       <c r="N722" t="b">
         <v>0</v>
@@ -29126,7 +29126,7 @@
         <v>886</v>
       </c>
       <c r="K727">
-        <v>32.946</v>
+        <v>32946</v>
       </c>
       <c r="N727" t="b">
         <v>0</v>
@@ -29155,7 +29155,7 @@
         <v>886</v>
       </c>
       <c r="K728">
-        <v>2.946</v>
+        <v>2946</v>
       </c>
       <c r="N728" t="b">
         <v>0</v>
@@ -29184,7 +29184,7 @@
         <v>886</v>
       </c>
       <c r="K729">
-        <v>2.946</v>
+        <v>2946</v>
       </c>
       <c r="N729" t="b">
         <v>0</v>
@@ -29216,7 +29216,7 @@
         <v>886</v>
       </c>
       <c r="K730">
-        <v>7.866</v>
+        <v>7866</v>
       </c>
       <c r="N730" t="b">
         <v>0</v>
@@ -29248,7 +29248,7 @@
         <v>886</v>
       </c>
       <c r="K731">
-        <v>28.934</v>
+        <v>28934</v>
       </c>
       <c r="N731" t="b">
         <v>0</v>
@@ -29423,7 +29423,7 @@
         <v>886</v>
       </c>
       <c r="K736">
-        <v>32.048</v>
+        <v>32048</v>
       </c>
       <c r="N736" t="b">
         <v>0</v>
@@ -29452,7 +29452,7 @@
         <v>886</v>
       </c>
       <c r="K737">
-        <v>2.048</v>
+        <v>2048</v>
       </c>
       <c r="N737" t="b">
         <v>0</v>
@@ -29481,7 +29481,7 @@
         <v>886</v>
       </c>
       <c r="K738">
-        <v>2.048</v>
+        <v>2048</v>
       </c>
       <c r="N738" t="b">
         <v>0</v>
@@ -29513,7 +29513,7 @@
         <v>886</v>
       </c>
       <c r="K739">
-        <v>32.048</v>
+        <v>32048</v>
       </c>
       <c r="N739" t="b">
         <v>0</v>
@@ -29545,7 +29545,7 @@
         <v>886</v>
       </c>
       <c r="K740">
-        <v>32.048</v>
+        <v>32048</v>
       </c>
       <c r="N740" t="b">
         <v>0</v>
@@ -29720,7 +29720,7 @@
         <v>886</v>
       </c>
       <c r="K745">
-        <v>38.957</v>
+        <v>38957</v>
       </c>
       <c r="N745" t="b">
         <v>0</v>
@@ -29749,7 +29749,7 @@
         <v>886</v>
       </c>
       <c r="K746">
-        <v>8.946999999999999</v>
+        <v>8947</v>
       </c>
       <c r="N746" t="b">
         <v>0</v>
@@ -29778,7 +29778,7 @@
         <v>886</v>
       </c>
       <c r="K747">
-        <v>8.946999999999999</v>
+        <v>8947</v>
       </c>
       <c r="N747" t="b">
         <v>0</v>
@@ -29810,7 +29810,7 @@
         <v>886</v>
       </c>
       <c r="K748">
-        <v>32.152</v>
+        <v>32152</v>
       </c>
       <c r="N748" t="b">
         <v>0</v>
@@ -29842,7 +29842,7 @@
         <v>886</v>
       </c>
       <c r="K749">
-        <v>32.152</v>
+        <v>32152</v>
       </c>
       <c r="N749" t="b">
         <v>0</v>

</xml_diff>